<commit_message>
2-layer PRODUCTION: final JLCPCB + Lion Circuits release (wall sensors only)
Production-ready release for the 2-layer micromouse board (wall sensors
only, no line array/mux/JTAG): U8 (IMU) + U2 (motor driver) flipped to
the bottom layer, full clean-slate Freerouting re-route, GND pour
fragment bridging, BOM duplicate-part merge, and DRC cleanup (0 errors,
0 warnings). Includes matching production folders for both JLCPCB and
Lion Circuits (BOM, CPL, gerbers).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/JLCPCB_2layers/design/fab_release/jlcpcb/BOM_JLC-assembly.xlsx
+++ b/pcb/JLCPCB_2layers/design/fab_release/jlcpcb/BOM_JLC-assembly.xlsx
@@ -204,7 +204,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">C178588</t>
+          <t xml:space="preserve">C2887273</t>
         </is>
       </c>
     </row>
@@ -238,7 +238,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">D23,D24,D25,D26,D27,D28</t>
+          <t xml:space="preserve">D23,D24,D25,D26,D27,D28,D30,D31,D33</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -277,254 +277,254 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power LED 0603 red</t>
+          <t xml:space="preserve">WS2812B addressable RGB 5050</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">D30</t>
+          <t xml:space="preserve">D32</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_0603_1608Metric</t>
+          <t xml:space="preserve">LED_WS2812B_PLCC4_5.0x5.0mm_P3.2mm</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2286</t>
+          <t xml:space="preserve">C2843785</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status LED 0603 red</t>
+          <t xml:space="preserve">2.6A/16V PPTC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">D31</t>
+          <t xml:space="preserve">F1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_0603_1608Metric</t>
+          <t xml:space="preserve">Fuse_1812_4532Metric</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2286</t>
+          <t xml:space="preserve">C16490</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">WS2812B addressable RGB 5050</t>
+          <t xml:space="preserve">BATT_IN_2S</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">D32</t>
+          <t xml:space="preserve">J1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_WS2812B_PLCC4_5.0x5.0mm_P3.2mm</t>
+          <t xml:space="preserve">JST_XH_B2B-XH-A_1x02_P2.50mm_Vertical</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2761795</t>
+          <t xml:space="preserve">C158012</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motor-power LED 0603</t>
+          <t xml:space="preserve">MOTOR_A_N20_ENCODER</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">D33</t>
+          <t xml:space="preserve">J5,J6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_0603_1608Metric</t>
+          <t xml:space="preserve">JST_ZH_B6B-ZR_1x06_P1.50mm_Vertical</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2286</t>
+          <t xml:space="preserve">C157984</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.6A/16V PPTC</t>
+          <t xml:space="preserve">USB-C rear</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">F1</t>
+          <t xml:space="preserve">J7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuse_1812_4532Metric</t>
+          <t xml:space="preserve">USB_C_Receptacle_GCT_USB4105-xx-A_16P_TopMnt_Horizontal</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">C883162</t>
+          <t xml:space="preserve">C3020560</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATT_IN_2S</t>
+          <t xml:space="preserve">BATT_IN_XT60</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">J1</t>
+          <t xml:space="preserve">J10</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">JST_XH_B2B-XH-A_1x02_P2.50mm_Vertical</t>
+          <t xml:space="preserve">AMASS_XT60-M_1x02_P7.20mm_Vertical</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">C158012</t>
+          <t xml:space="preserve">C98733</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">MOTOR_A_N20_ENCODER</t>
+          <t xml:space="preserve">4.7uH</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">J5</t>
+          <t xml:space="preserve">L1,L2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">JST_ZH_B6B-ZR_1x06_P1.50mm_Vertical</t>
+          <t xml:space="preserve">L_Bourns_SRP4020TA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">C157984</t>
+          <t xml:space="preserve">C2041623</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">MOTOR_B_N20_ENCODER</t>
+          <t xml:space="preserve">Q_PMOS reverse guard</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">J6</t>
+          <t xml:space="preserve">Q1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">JST_ZH_B6B-ZR_1x06_P1.50mm_Vertical</t>
+          <t xml:space="preserve">SOT-23</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">C157984</t>
+          <t xml:space="preserve">C150492</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">USB-C rear</t>
+          <t xml:space="preserve">PT334-6B</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">J7</t>
+          <t xml:space="preserve">Q2,Q3,Q4,Q5,Q6,Q7</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">USB_C_Receptacle_GCT_USB4105-xx-A_16P_TopMnt_Horizontal</t>
+          <t xml:space="preserve">LED_D5.0mm_IRBlack</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">C3020560</t>
+          <t xml:space="preserve">C369188</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">BATT_IN_XT60</t>
+          <t xml:space="preserve">BSS138</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">J10</t>
+          <t xml:space="preserve">Q16,Q17,Q18</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMASS_XT60-M_1x02_P7.20mm_Vertical</t>
+          <t xml:space="preserve">SOT-23</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">C98733</t>
+          <t xml:space="preserve">C82045</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7uH</t>
+          <t xml:space="preserve">BSS84</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">L1,L2</t>
+          <t xml:space="preserve">Q28,Q29,Q30,Q31,Q32,Q33</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">L_Bourns_SRP4020TA</t>
+          <t xml:space="preserve">SOT-23</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2041623</t>
+          <t xml:space="preserve">C82079</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q_PMOS reverse guard</t>
+          <t xml:space="preserve">MMBT2222A</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q1</t>
+          <t xml:space="preserve">Q34</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -534,107 +534,107 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">C150492</t>
+          <t xml:space="preserve">C94515</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT334-6B</t>
+          <t xml:space="preserve">100k</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2,Q3,Q4,Q5,Q6,Q7</t>
+          <t xml:space="preserve">R1,R2,R62,R63,R64,R69,R73</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED_D5.0mm_IRBlack</t>
+          <t xml:space="preserve">R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">C369188</t>
+          <t xml:space="preserve">C96346</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSS138</t>
+          <t xml:space="preserve">39k</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q16,Q17,Q18</t>
+          <t xml:space="preserve">R3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23</t>
+          <t xml:space="preserve">R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">C82045</t>
+          <t xml:space="preserve">C113306</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSS84</t>
+          <t xml:space="preserve">10k</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q28,Q29,Q30,Q31,Q32,Q33</t>
+          <t xml:space="preserve">R6,R7,R8,R9,R10,R11,R55,R65,R67,R79,R80</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23</t>
+          <t xml:space="preserve">R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">C82079</t>
+          <t xml:space="preserve">C108451</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMBT2222A</t>
+          <t xml:space="preserve">5.1k</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q34</t>
+          <t xml:space="preserve">R12,R56</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23</t>
+          <t xml:space="preserve">R_0805_2012Metric</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">C94515</t>
+          <t xml:space="preserve">C27834</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">100k</t>
+          <t xml:space="preserve">47k</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">R1,R2,R62,R63,R64,R69,R73</t>
+          <t xml:space="preserve">R13,R15,R17,R19,R21,R23</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -644,19 +644,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">C96346</t>
+          <t xml:space="preserve">C17713</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">39k</t>
+          <t xml:space="preserve">33</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">R3</t>
+          <t xml:space="preserve">R14,R16,R18,R20,R22,R24</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -666,19 +666,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">C113306</t>
+          <t xml:space="preserve">C17634</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">10k</t>
+          <t xml:space="preserve">1k</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">R6,R7,R8,R9,R10,R11,R55,R65,R67,R79,R80</t>
+          <t xml:space="preserve">R49,R50,R51,R52,R53,R54,R57,R58,R82,R83,R84</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -688,19 +688,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17414</t>
+          <t xml:space="preserve">C17513</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.1k</t>
+          <t xml:space="preserve">15k</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">R12,R56</t>
+          <t xml:space="preserve">R68</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -710,19 +710,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">C27834</t>
+          <t xml:space="preserve">C17475</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">47k</t>
+          <t xml:space="preserve">220k</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">R13,R15,R17,R19,R21,R23</t>
+          <t xml:space="preserve">R70</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -732,19 +732,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17713</t>
+          <t xml:space="preserve">C17556</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">33</t>
+          <t xml:space="preserve">110k</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">R14,R16,R18,R20,R22,R24</t>
+          <t xml:space="preserve">R71</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -754,19 +754,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17634</t>
+          <t xml:space="preserve">C2907221</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">1k</t>
+          <t xml:space="preserve">11k</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">R49,R50,R51,R52,R53,R54,R57,R58,R82,R83,R84</t>
+          <t xml:space="preserve">R74</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17513</t>
+          <t xml:space="preserve">C17429</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">15k</t>
+          <t xml:space="preserve">4.7k</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">R68</t>
+          <t xml:space="preserve">R77,R78</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -798,19 +798,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17475</t>
+          <t xml:space="preserve">C17673</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">220k</t>
+          <t xml:space="preserve">220</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">R70</t>
+          <t xml:space="preserve">R81</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -820,357 +820,181 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17556</t>
+          <t xml:space="preserve">C17557</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">110k</t>
+          <t xml:space="preserve">Tactile pushbutton switch</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">R71</t>
+          <t xml:space="preserve">SW1,SW2,SW3,SW4</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">SW_Push_1P1T_NO_CK_KMR2</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2907221</t>
+          <t xml:space="preserve">C269272</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">11k</t>
+          <t xml:space="preserve">PWR ALL</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">R74</t>
+          <t xml:space="preserve">SW5,SW6</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">SW_SPDT_PCM12</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17429</t>
+          <t xml:space="preserve">C221841</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7k</t>
+          <t xml:space="preserve">AP63203WU-7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">R77,R78</t>
+          <t xml:space="preserve">U1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">TSOT-23-6</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17673</t>
+          <t xml:space="preserve">C780769</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">220</t>
+          <t xml:space="preserve">TB6612FNG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">R81</t>
+          <t xml:space="preserve">U2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">R_0805_2012Metric</t>
+          <t xml:space="preserve">SSOP-24_5.3x8.2mm_P0.65mm</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17557</t>
+          <t xml:space="preserve">C141517</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">BTN_A</t>
+          <t xml:space="preserve">ESP32-S3-WROOM-1-N8R2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW1</t>
+          <t xml:space="preserve">U3</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW_PUSH_6mm</t>
+          <t xml:space="preserve">ESP32-S3-WROOM-1</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">C285524</t>
+          <t xml:space="preserve">C2913204</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">RESET</t>
+          <t xml:space="preserve">USBLC6-2SC6</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW2</t>
+          <t xml:space="preserve">U6</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW_PUSH_6mm</t>
+          <t xml:space="preserve">SOT-23-6</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">C285524</t>
+          <t xml:space="preserve">C7519</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">BTN_B</t>
+          <t xml:space="preserve">TPS54302DDCR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW3</t>
+          <t xml:space="preserve">U7</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW_PUSH_6mm</t>
+          <t xml:space="preserve">SOT-23-6</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">C285524</t>
+          <t xml:space="preserve">C311983</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">BTN_C</t>
+          <t xml:space="preserve">BNO055</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW4</t>
+          <t xml:space="preserve">U8</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">SW_PUSH_6mm</t>
+          <t xml:space="preserve">BNO055</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C285524</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PWR ALL</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW5</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_SPDT_PCM12</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C221841</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PWR MOTORS</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW6</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_SPDT_PCM12</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C221841</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AP63203WU-7</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U1</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TSOT-23-6</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C780769</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TB6612FNG</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U2</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SSOP-24_5.3x8.2mm_P0.65mm</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C141517</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ESP32-S3-WROOM-1-N8R2</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U3</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ESP32-S3-WROOM-1</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C2913204</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USBLC6-2SC6</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U6</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOT-23-6</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C7519</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TPS54302DDCR</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U7</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOT-23-6</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C311983</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BNO055</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U8</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BNO055</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
         <is>
           <t xml:space="preserve">C93216</t>
         </is>

</xml_diff>